<commit_message>
chore(F132): civil services loader, validators, agents, docs; F132 marked Done
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ExamPrep_AI_Module_Development_Plan.xlsx
+++ b/docs/ExamPrep_AI_Module_Development_Plan.xlsx
@@ -1,29 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="760" yWindow="760" windowWidth="14400" windowHeight="7270" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00 Read Me" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Product Scope" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 Module Master" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 Feature Backlog" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Data Model" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 API Endpoints" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Screens &amp; Routes" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 AI Layer" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Gap Analysis" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Tech Stack" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Roadmap" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 Risks" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 QA &amp; Test Plan" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 Effort Summary" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14 Competitive Benchmark" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15 Capability Matrix" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16 Question Bank Plan" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17 Rollout Sequence" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="00 Read Me" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="01 Product Scope" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="02 Module Master" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="03 Feature Backlog" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="04 Data Model" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="05 API Endpoints" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="06 Screens &amp; Routes" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="07 AI Layer" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="08 Gap Analysis" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="09 Tech Stack" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="10 Roadmap" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="11 Risks" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="12 QA &amp; Test Plan" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="13 Effort Summary" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="14 Competitive Benchmark" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="15 Capability Matrix" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="16 Question Bank Plan" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="17 Rollout Sequence" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01 Product Scope'!$A$3:$D$26</definedName>
@@ -10632,7 +10632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K134"/>
+  <dimension ref="A1:K135"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
     <col width="10" customWidth="1" style="38" min="1" max="2"/>
@@ -10649,7 +10649,7 @@
     <row r="1" ht="24" customHeight="1" s="38">
       <c r="A1" s="42" t="inlineStr">
         <is>
-          <t>03  Feature Backlog  —  131 features. Type Not Started / In Progress / Blocked / Done in column J.</t>
+          <t>03  Feature Backlog  —  132 features. Type Not Started / In Progress / Blocked / Done in column J.</t>
         </is>
       </c>
     </row>
@@ -17816,6 +17816,63 @@
       <c r="K134" t="inlineStr">
         <is>
           <t>Added 2026-09-30 at the owner's request, reversing tab 01's 'Native mobile apps: out of scope v1'. TWA, not a native rewrite (owner approved): every web feature ships on day one and web deploys reach the app without a Play update. Owner arranging: personal Play Console account (needs a 12-tester, 14-day closed test before production) and a custom domain (the app is bound to its domain, so this must be set before the first Play upload). 2026-09-30 later, owner decisions: domain www.prepplan.in (registered at GoDaddy; the apex redirects to www), Android appId in.prepplan.app (permanent), user-facing brand renamed ExamPrep AI -&gt; PrepPlan across web + app (internal names unchanged), support email support@prepplan.in. Also added public /privacy and /delete-account pages and docs/android/play-console-answers.md. Open blocker: a student who signed up alone cannot delete her own account.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="15" customHeight="1" s="38">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>M05</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>F132</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>UPSC Civil Services Prelims - Indian Polity question bank (Laxmikanth, trend-based)</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>As a civil services aspirant I want polity practice questions written in the style UPSC Prelims uses now (multi-statement, how-many, Statement-I/II), each traceable to a Laxmikanth page, so that my practice matches the exam and not a recall quiz.</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Subject POLITY, board CIVILS, class 0, concept codes LK-&lt;chapter&gt;.&lt;n&gt; mapped to Laxmikanth, Indian Polity 8e. Every concept holds 20 approved questions in the 2020-26 trend mix (about 25% direct, 45% which-statements, 15% how-many, 10% Statement-I/II, 5% match); every question carries an explanation, a reason each wrong option fails and a source page; every pack has passed an independent review with no HIGH finding; options are shuffled at load; the previous one-line questions are retired, never deleted; past-year questions and trend report live in content/authoring/civil/polity and docs/CIVIL_SERVICES_POLITY_*.md.</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G135" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H135" s="10" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>S23</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>Added 2026-10-09 at the owner's request. Polity only (History, Geography, Economy get their own agents later). Agents civil-polity-author / civil-polity-reviewer; loader scripts/load-civil-pack.ts. Status and open items: docs/CIVIL_SERVICES_POLITY_STATUS.md. Production load and retiring the old 2,500 questions need the owner's explicit go-ahead. | 2026-10-12: Laxmikanth set (4,160), AKS study-notes set (2,120) and upgraded NCERT-style chapters I1-I4/II1 (660) loaded to production; old 660 retired; 20 approved per concept verified. See docs/CIVIL_SERVICES_POLITY_STATUS.md.</t>
         </is>
       </c>
     </row>
@@ -17825,7 +17882,7 @@
     <mergeCell ref="A1:K1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="J4:J134" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J4:J135" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Started,In Progress,Blocked,Done"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>